<commit_message>
Fix critical security flaws: prevent unauthorized access, add route-level authorization, fix admin-first auth logic
</commit_message>
<xml_diff>
--- a/Resident PII Test.xlsx
+++ b/Resident PII Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://us-partner-integrations.egnyte.com/msoffice/wopi/files/74150128-3130-449b-9442-02fce02f5e8e/WOPIServiceId_TP_EGNYTE_PLUS/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_6949D2B9D340D71DB5E1D2F0505ED87656C6EB93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBDF47B6-4681-4EBF-A8BB-C037E30AFCA6}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_6949D2B9D340D71DB5E1D2F0505ED87656C6EB93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC75EBB3-BCFA-4A39-B42F-CFE4C5E804F7}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20135,7 +20135,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -20148,6 +20148,14 @@
       <color rgb="FF323130"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -20167,14 +20175,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -20481,6 +20492,7 @@
     <col min="1" max="1" width="21.5703125" customWidth="1"/>
     <col min="2" max="2" width="25.85546875" customWidth="1"/>
     <col min="6" max="6" width="23.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -20601,7 +20613,7 @@
       <c r="A4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>6700</v>
       </c>
       <c r="C4" t="s">
@@ -58523,6 +58535,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L1001" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{29A7D63A-F335-4F0E-8CA5-5AEBE2520368}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>